<commit_message>
debrecen és baja ip cím excel
</commit_message>
<xml_diff>
--- a/IP címek.xlsx
+++ b/IP címek.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rafael\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECA151EE-1245-45C4-B585-E480A6486376}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BABAE0B-A811-4540-8278-34A0D08A95EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bajai telephely (Központ)" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="212">
   <si>
     <t>Helyiség</t>
   </si>
@@ -50,9 +50,6 @@
     <t>Port</t>
   </si>
   <si>
-    <t>IP cím</t>
-  </si>
-  <si>
     <t>Tárgyaló</t>
   </si>
   <si>
@@ -239,9 +236,6 @@
     <t>DHCP</t>
   </si>
   <si>
-    <t>DHCP 10.10.100.64/27</t>
-  </si>
-  <si>
     <t>Győr_SW1</t>
   </si>
   <si>
@@ -296,15 +290,6 @@
     <t>targyalo_sw2</t>
   </si>
   <si>
-    <t>targyalo_wireless1</t>
-  </si>
-  <si>
-    <t>targyalo_wireless2</t>
-  </si>
-  <si>
-    <t>targyalo_wireless3</t>
-  </si>
-  <si>
     <t>targyalo_tablet1</t>
   </si>
   <si>
@@ -314,18 +299,12 @@
     <t>targyalo_laptop</t>
   </si>
   <si>
-    <t>DHCP 10.10.100.1/27</t>
-  </si>
-  <si>
     <t>Nyomtato_RG</t>
   </si>
   <si>
     <t>10.10.100.3</t>
   </si>
   <si>
-    <t>DHCP 10.10.100.128/27</t>
-  </si>
-  <si>
     <t>Nyomtato_Iroda1</t>
   </si>
   <si>
@@ -350,9 +329,6 @@
     <t>Telefon_iroda4</t>
   </si>
   <si>
-    <t>DHCP 10.10.100.32/27</t>
-  </si>
-  <si>
     <t>HQ_Router</t>
   </si>
   <si>
@@ -488,9 +464,6 @@
     <t>Dualstack</t>
   </si>
   <si>
-    <t>Ipv6</t>
-  </si>
-  <si>
     <t>Ipv4</t>
   </si>
   <si>
@@ -521,9 +494,6 @@
     <t>172.16.100.33/27</t>
   </si>
   <si>
-    <t>172.16.100.97/26</t>
-  </si>
-  <si>
     <t>172.16.100.225/27</t>
   </si>
   <si>
@@ -539,30 +509,6 @@
     <t>ipv6 add 2001:db8:acad:c::1/64</t>
   </si>
   <si>
-    <t>(DHCP) 172.16.100.129/27</t>
-  </si>
-  <si>
-    <t>(DHCP) 172.16.100.129/28</t>
-  </si>
-  <si>
-    <t>(DHCP) 172.16.100.129/29</t>
-  </si>
-  <si>
-    <t>(DHCP) 172.16.100.129/30</t>
-  </si>
-  <si>
-    <t>SLAAC (ipv6 add 2001:db8:acad:d::1/64)</t>
-  </si>
-  <si>
-    <t>stateful DHCP (ipv6 add 2001:db8:acad:b::1/64)</t>
-  </si>
-  <si>
-    <t>stateless DHCP (ipv6 add 2001:db8:acad:a::1/64)</t>
-  </si>
-  <si>
-    <t>SLAAC (ipv6 add 2001:db8:acad:c::1/64)</t>
-  </si>
-  <si>
     <t>172.16.100.35/27</t>
   </si>
   <si>
@@ -575,15 +521,6 @@
     <t>172.16.100.67/27</t>
   </si>
   <si>
-    <t>172.16.100.68/28</t>
-  </si>
-  <si>
-    <t>172.16.100.69/28</t>
-  </si>
-  <si>
-    <t>172.16.100.70/29</t>
-  </si>
-  <si>
     <t>172.16.100.98/27</t>
   </si>
   <si>
@@ -591,13 +528,160 @@
   </si>
   <si>
     <t>172.16.100.100/27</t>
+  </si>
+  <si>
+    <t>ipv6</t>
+  </si>
+  <si>
+    <t>Stateful DHCP</t>
+  </si>
+  <si>
+    <t>Stateless DHCP</t>
+  </si>
+  <si>
+    <t>ipv4</t>
+  </si>
+  <si>
+    <t>Statikus</t>
+  </si>
+  <si>
+    <t>Dinamikus</t>
+  </si>
+  <si>
+    <t>172.16.100.130/27</t>
+  </si>
+  <si>
+    <t>172.16.100.131/27</t>
+  </si>
+  <si>
+    <t>172.16.100.132/27</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 172.16.100.132/27</t>
+  </si>
+  <si>
+    <t>2001:db8:acad:d::1/64</t>
+  </si>
+  <si>
+    <t>2001:db8:acad:a::1/64</t>
+  </si>
+  <si>
+    <t>2001:db8:acad:c::1/64</t>
+  </si>
+  <si>
+    <t>172.16.100.68/27</t>
+  </si>
+  <si>
+    <t>172.16.100.69/27</t>
+  </si>
+  <si>
+    <t>172.16.100.70/27</t>
+  </si>
+  <si>
+    <t>172.16.100.97/27</t>
+  </si>
+  <si>
+    <t>2001:db8:acad:b::1/64</t>
+  </si>
+  <si>
+    <t>172.16.100.101/27</t>
+  </si>
+  <si>
+    <t>10.10.100.100</t>
+  </si>
+  <si>
+    <t>targyalo_wireless</t>
+  </si>
+  <si>
+    <t>piheno_wireless</t>
+  </si>
+  <si>
+    <t>recepcio_wireless</t>
+  </si>
+  <si>
+    <t>10.10.100.101</t>
+  </si>
+  <si>
+    <t>10.10.100.102</t>
+  </si>
+  <si>
+    <t>Baja_WLC</t>
+  </si>
+  <si>
+    <t>gig1</t>
+  </si>
+  <si>
+    <t>10.10.100.99</t>
+  </si>
+  <si>
+    <t>10.10.100.64/27</t>
+  </si>
+  <si>
+    <t>10.10.100.96/27</t>
+  </si>
+  <si>
+    <t>10.10.100.128/27</t>
+  </si>
+  <si>
+    <t>10.10.100.32/27</t>
+  </si>
+  <si>
+    <t>10.10.100.1/27</t>
+  </si>
+  <si>
+    <t>Kozponti_router</t>
+  </si>
+  <si>
+    <t>g1/0/1</t>
+  </si>
+  <si>
+    <t>g1/0/2</t>
+  </si>
+  <si>
+    <t>g1/0/3</t>
+  </si>
+  <si>
+    <t>g1/0/4</t>
+  </si>
+  <si>
+    <t>g1/0/5</t>
+  </si>
+  <si>
+    <t>10.10.100.33/27</t>
+  </si>
+  <si>
+    <t>10.10.100.65/27</t>
+  </si>
+  <si>
+    <t>10.10.100.97/27</t>
+  </si>
+  <si>
+    <t>10.10.100.129/27</t>
+  </si>
+  <si>
+    <t>10.10.30.6/27</t>
+  </si>
+  <si>
+    <t>RG_router</t>
+  </si>
+  <si>
+    <t>g0/0/0</t>
+  </si>
+  <si>
+    <t>s0/1/0</t>
+  </si>
+  <si>
+    <t>10.10.30.5/27</t>
+  </si>
+  <si>
+    <t>75.92.210.10/30</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -611,6 +695,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -620,7 +719,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -840,24 +939,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
@@ -867,11 +975,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normál" xfId="0" builtinId="0"/>
@@ -1186,374 +1316,596 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8263A6BB-B1A9-48B3-9C01-A0B104726D87}">
-  <dimension ref="A3:D40"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.33203125" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="16.44140625" customWidth="1"/>
     <col min="4" max="4" width="28.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="12" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D1" s="35" t="s">
+        <v>141</v>
+      </c>
+      <c r="E1" s="35"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B2" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C2" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D2" s="28" t="s">
+        <v>167</v>
+      </c>
+      <c r="E2" s="28" t="s">
+        <v>168</v>
+      </c>
+      <c r="H2" s="25"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="27" t="s">
+        <v>81</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B4" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B5" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B6" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B7" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="31" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="8" t="s">
+      <c r="B9" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C10" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C11" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C12" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C13" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B14" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="C14" s="22" t="s">
+        <v>208</v>
+      </c>
+      <c r="D14" s="22" t="s">
+        <v>195</v>
+      </c>
+      <c r="E14" s="5"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C15" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="D15" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="E15" s="5"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C16" s="22" t="s">
+        <v>209</v>
+      </c>
+      <c r="D16" s="22" t="s">
+        <v>211</v>
+      </c>
+      <c r="E16" s="5"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B18" s="22" t="s">
+        <v>188</v>
+      </c>
+      <c r="C18" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B19" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="E19" s="24" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B20" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="E20" s="17" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B21" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B22" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="E22" s="17" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B23" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B5" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B6" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B7" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B8" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" s="1" t="s">
+      <c r="C23" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D23" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B24" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B10" s="1" t="s">
+      <c r="C24" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D24" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B25" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="1"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B11" s="1" t="s">
+      <c r="C25" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D25" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" s="27" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D31" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B32" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D32" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B33" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D33" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D35" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B36" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D36" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B37" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D37" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B38" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D38" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B39" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D39" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B40" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D40" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B41" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D41" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B42" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D42" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B43" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D43" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B44" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D44" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B45" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D45" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B46" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D46" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D48" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="49" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B49" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" s="2"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B12" s="1" t="s">
+      <c r="C49" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D49" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E49" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="50" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B50" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D50" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="51" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B51" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D51" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="1"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D13" s="2"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B14" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D14" s="1"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B15" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D15" s="1"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B19" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B20" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B24" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B25" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B26" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B27" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B28" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B29" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B30" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B31" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B32" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B33" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B34" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A37" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B38" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B39" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B40" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D40" s="1" t="s">
-        <v>93</v>
+      <c r="E51" s="17" t="s">
+        <v>144</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="D1:E1"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1570,271 +1922,271 @@
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C2" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="1" t="s">
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C3" s="6"/>
+      <c r="D3" s="3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C3" s="7"/>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E3" s="1" t="s">
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C4" s="6"/>
+      <c r="D4" s="4" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C4" s="7"/>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="2" t="s">
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C5" s="6"/>
+      <c r="D5" s="5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C5" s="7"/>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="5" t="s">
         <v>35</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C7" s="5" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C10" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>60</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E11" s="1" t="s">
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B12" s="6"/>
+      <c r="C12" s="4" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B12" s="7"/>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" s="2" t="s">
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B13" s="6"/>
+      <c r="C13" s="4" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B13" s="7"/>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C14" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>45</v>
-      </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B16" s="8" t="s">
-        <v>17</v>
+      <c r="B16" s="7" t="s">
+        <v>16</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C17" s="5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C18" s="5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C19" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E19" s="5" t="s">
         <v>46</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C20" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C21" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C22" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22" s="5" t="s">
         <v>50</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C23" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E23" s="5" t="s">
         <v>52</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C24" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B27" s="8" t="s">
-        <v>13</v>
+      <c r="B27" s="7" t="s">
+        <v>12</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C28" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="D28" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="E28" s="10" t="s">
-        <v>65</v>
+      <c r="C28" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C29" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C30" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C31" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1845,350 +2197,500 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5745176A-E3EE-4736-AEBC-6021C2097FDE}">
-  <dimension ref="A2:E27"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="29.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="40.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="23" customWidth="1"/>
+    <col min="5" max="5" width="41.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.88671875" customWidth="1"/>
+    <col min="7" max="7" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="41.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D2" s="20" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D1" s="35" t="s">
+        <v>140</v>
+      </c>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D2" s="35" t="s">
+        <v>163</v>
+      </c>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="36" t="s">
+        <v>166</v>
+      </c>
+      <c r="H2" s="20"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="27" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="28" t="s">
+        <v>167</v>
+      </c>
+      <c r="E3" s="28" t="s">
+        <v>164</v>
+      </c>
+      <c r="F3" s="28" t="s">
+        <v>165</v>
+      </c>
+      <c r="G3" s="28" t="s">
+        <v>167</v>
+      </c>
+      <c r="H3" s="21"/>
+      <c r="I3" s="19"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="31" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="31" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>142</v>
+      </c>
+      <c r="D4" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="E4" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="F4" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C5" s="30" t="s">
+        <v>145</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="E5" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="F5" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C6" s="30" t="s">
+        <v>146</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E6" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="F6" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C7" s="30" t="s">
+        <v>147</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="E7" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="F7" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="I7" s="19"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C8" s="30" t="s">
         <v>148</v>
       </c>
-      <c r="E2" s="20"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="5" t="s">
+      <c r="D8" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E8" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="F8" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C9" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="16" t="s">
-        <v>151</v>
-      </c>
-      <c r="D4" s="19" t="s">
-        <v>153</v>
-      </c>
-      <c r="E4" s="5" t="s">
+      <c r="D9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="F9" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C5" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="E5" s="5" t="s">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B10" s="31" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="E10" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B11" s="31" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="E11" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B12" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="E12" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B13" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="E13" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="31" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="32" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="F14" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="G14" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="J14" s="18" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="25"/>
+      <c r="B15" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="F15" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="G15" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" s="31" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="E16" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="G16" s="5" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C6" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="E6" s="5" t="s">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B17" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="E17" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="G17" s="5" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C7" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="E7" s="5" t="s">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B18" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="E18" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B19" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="E19" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B20" s="31" t="s">
+        <v>21</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="E20" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="F21" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="G21" s="5" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C8" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="D8" s="19" t="s">
-        <v>153</v>
-      </c>
-      <c r="E8" s="5" t="s">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B22" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="F22" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="G22" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C9" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E9" s="5" t="s">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B23" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D23" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="F23" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="G23" s="5" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B10" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B11" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C11" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B12" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="E12" s="21" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B13" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C15" s="21" t="s">
-        <v>9</v>
-      </c>
-      <c r="D15" s="21" t="s">
-        <v>171</v>
-      </c>
-      <c r="E15" s="21" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="12"/>
-      <c r="B16" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="E16" s="5" t="s">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B24" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D24" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="E24" s="5" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="22"/>
-      <c r="B17" s="22"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C19" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B20" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="D20" s="21" t="s">
-        <v>172</v>
-      </c>
-      <c r="E20" s="21" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B21" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B22" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B23" s="22"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="E24" s="5" t="s">
+      <c r="F24" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="G24" s="5" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B25" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B26" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B27" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="E27" s="5"/>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D25" s="25"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="25"/>
+      <c r="G25" s="25"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="D2:E2"/>
+  <mergeCells count="2">
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="D1:G1"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2208,283 +2710,283 @@
   <sheetData>
     <row r="2" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C2" s="5" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C3" s="7"/>
+      <c r="C3" s="6"/>
       <c r="D3" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C4" s="7"/>
+      <c r="C4" s="6"/>
       <c r="D4" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C5" s="7"/>
+      <c r="C5" s="6"/>
     </row>
     <row r="7" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C7" s="5" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" spans="3:5" x14ac:dyDescent="0.3">
       <c r="D8" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
     </row>
     <row r="10" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C10" s="13" t="s">
-        <v>112</v>
+      <c r="C10" s="11" t="s">
+        <v>104</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" spans="3:5" x14ac:dyDescent="0.3">
       <c r="D11" s="5" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" spans="3:5" x14ac:dyDescent="0.3">
       <c r="D12" s="5" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13" spans="3:5" x14ac:dyDescent="0.3">
       <c r="D13" s="5" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
     </row>
     <row r="14" spans="3:5" x14ac:dyDescent="0.3">
       <c r="D14" s="5" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
     </row>
     <row r="15" spans="3:5" x14ac:dyDescent="0.3">
       <c r="D15" s="5" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C18" s="1" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B19" s="7"/>
+      <c r="B19" s="6"/>
       <c r="C19" s="4" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B20" s="7"/>
+      <c r="B20" s="6"/>
       <c r="C20" s="4" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C21" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B23" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="D21" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B23" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>139</v>
-      </c>
       <c r="D23" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C24" s="5" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C25" s="5" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B27" s="5" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C28" s="15" t="s">
-        <v>146</v>
+      <c r="C28" s="13" t="s">
+        <v>138</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.3">
       <c r="C29" s="5" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B32" s="8" t="s">
-        <v>13</v>
+      <c r="B32" s="7" t="s">
+        <v>12</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
     </row>
     <row r="33" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C33" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="D33" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="E33" s="10" t="s">
-        <v>65</v>
+        <v>128</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="34" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="C34" s="11" t="s">
-        <v>135</v>
+      <c r="C34" s="10" t="s">
+        <v>127</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="35" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C35" s="5" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>